<commit_message>
feat: suporte a múltiplos filtros, novas categorias e ajustes visuais
</commit_message>
<xml_diff>
--- a/Planilha Cris.xlsx
+++ b/Planilha Cris.xlsx
@@ -28040,9 +28040,6 @@
       <c r="A1" t="str">
         <v xml:space="preserve">Condomínio do Edif. Acary </v>
       </c>
-      <c r="H1" t="str">
-        <v>COBRANÇA AGUA</v>
-      </c>
       <c r="I1" t="str">
         <v>COBRANÇA: ÁGUA</v>
       </c>
@@ -28146,6 +28143,36 @@
       </c>
       <c r="T6" t="str">
         <v>PAGO</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="T7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="T8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="T11" t="str">
+        <v>PG</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="T12" t="str">
+        <v>PG</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="T14" t="str">
+        <v>PG</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="T22" t="str">
+        <v>PG</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: calcular faturamento de todas as notas e entrada apenas de faturas pagas
</commit_message>
<xml_diff>
--- a/Planilha Cris.xlsx
+++ b/Planilha Cris.xlsx
@@ -28146,28 +28146,371 @@
       </c>
     </row>
     <row r="7">
+      <c r="A7" t="str">
+        <v>Janeiro</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2024</v>
+      </c>
+      <c r="C7" t="str">
+        <v>1</v>
+      </c>
+      <c r="D7" t="str">
+        <v>100,00</v>
+      </c>
+      <c r="E7" t="str">
+        <v>80</v>
+      </c>
+      <c r="F7" t="str">
+        <v>20</v>
+      </c>
+      <c r="G7" t="str">
+        <v>8.8</v>
+      </c>
+      <c r="H7" t="str">
+        <v>91.2</v>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
       <c r="T7" t="str">
         <v/>
       </c>
     </row>
     <row r="8">
+      <c r="A8" t="str">
+        <v>Fevereiro</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2024</v>
+      </c>
+      <c r="C8" t="str">
+        <v>2</v>
+      </c>
+      <c r="D8" t="str">
+        <v>100</v>
+      </c>
+      <c r="E8" t="str">
+        <v>80</v>
+      </c>
+      <c r="F8" t="str">
+        <v>20</v>
+      </c>
+      <c r="G8" t="str">
+        <v>8.8</v>
+      </c>
+      <c r="H8" t="str">
+        <v>91.2</v>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
       <c r="T8" t="str">
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Março</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2024</v>
+      </c>
+      <c r="C9" t="str">
+        <v>3</v>
+      </c>
+      <c r="D9" t="str">
+        <v>100</v>
+      </c>
+      <c r="E9" t="str">
+        <v>80</v>
+      </c>
+      <c r="F9" t="str">
+        <v>20</v>
+      </c>
+      <c r="G9" t="str">
+        <v>8.8</v>
+      </c>
+      <c r="H9" t="str">
+        <v>91.2</v>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Abril</v>
+      </c>
+      <c r="B10" t="str">
+        <v>2024</v>
+      </c>
+      <c r="C10" t="str">
+        <v>4</v>
+      </c>
+      <c r="D10" t="str">
+        <v>100</v>
+      </c>
+      <c r="E10" t="str">
+        <v>80</v>
+      </c>
+      <c r="F10" t="str">
+        <v>20</v>
+      </c>
+      <c r="G10" t="str">
+        <v>8.8</v>
+      </c>
+      <c r="H10" t="str">
+        <v>91.2</v>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+    </row>
     <row r="11">
+      <c r="A11" t="str">
+        <v>Maio</v>
+      </c>
+      <c r="B11" t="str">
+        <v>2024</v>
+      </c>
+      <c r="C11" t="str">
+        <v>5</v>
+      </c>
+      <c r="D11" t="str">
+        <v>100</v>
+      </c>
+      <c r="E11" t="str">
+        <v>80</v>
+      </c>
+      <c r="F11" t="str">
+        <v>20</v>
+      </c>
+      <c r="G11" t="str">
+        <v>8.8</v>
+      </c>
+      <c r="H11" t="str">
+        <v>91.2</v>
+      </c>
       <c r="T11" t="str">
         <v>PG</v>
       </c>
     </row>
     <row r="12">
+      <c r="A12" t="str">
+        <v>Junho</v>
+      </c>
+      <c r="B12" t="str">
+        <v>2024</v>
+      </c>
+      <c r="C12" t="str">
+        <v>6</v>
+      </c>
+      <c r="D12" t="str">
+        <v>100</v>
+      </c>
+      <c r="E12" t="str">
+        <v>80</v>
+      </c>
+      <c r="F12" t="str">
+        <v>20</v>
+      </c>
+      <c r="G12" t="str">
+        <v>8.8</v>
+      </c>
+      <c r="H12" t="str">
+        <v>91.2</v>
+      </c>
       <c r="T12" t="str">
         <v>PG</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Julho</v>
+      </c>
+      <c r="B13" t="str">
+        <v>2024</v>
+      </c>
+      <c r="C13" t="str">
+        <v>7</v>
+      </c>
+      <c r="D13" t="str">
+        <v>100</v>
+      </c>
+      <c r="E13" t="str">
+        <v>80</v>
+      </c>
+      <c r="F13" t="str">
+        <v>20</v>
+      </c>
+      <c r="G13" t="str">
+        <v>8.8</v>
+      </c>
+      <c r="H13" t="str">
+        <v>91.2</v>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+    </row>
     <row r="14">
+      <c r="A14" t="str">
+        <v>Agosto</v>
+      </c>
+      <c r="B14" t="str">
+        <v>2024</v>
+      </c>
+      <c r="C14" t="str">
+        <v>8</v>
+      </c>
+      <c r="D14" t="str">
+        <v>100</v>
+      </c>
+      <c r="E14" t="str">
+        <v>80</v>
+      </c>
+      <c r="F14" t="str">
+        <v>20</v>
+      </c>
+      <c r="G14" t="str">
+        <v>8.8</v>
+      </c>
+      <c r="H14" t="str">
+        <v>91.2</v>
+      </c>
       <c r="T14" t="str">
         <v>PG</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Setembro</v>
+      </c>
+      <c r="B15" t="str">
+        <v>2024</v>
+      </c>
+      <c r="C15" t="str">
+        <v>9</v>
+      </c>
+      <c r="D15" t="str">
+        <v>100</v>
+      </c>
+      <c r="E15" t="str">
+        <v>80</v>
+      </c>
+      <c r="F15" t="str">
+        <v>20</v>
+      </c>
+      <c r="G15" t="str">
+        <v>8.8</v>
+      </c>
+      <c r="H15" t="str">
+        <v>91.2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Outubro</v>
+      </c>
+      <c r="B16" t="str">
+        <v>2024</v>
+      </c>
+      <c r="C16" t="str">
+        <v>10</v>
+      </c>
+      <c r="D16" t="str">
+        <v>100</v>
+      </c>
+      <c r="E16" t="str">
+        <v>80</v>
+      </c>
+      <c r="F16" t="str">
+        <v>20</v>
+      </c>
+      <c r="G16" t="str">
+        <v>8.8</v>
+      </c>
+      <c r="H16" t="str">
+        <v>91.2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Novembro</v>
+      </c>
+      <c r="B17" t="str">
+        <v>2024</v>
+      </c>
+      <c r="C17" t="str">
+        <v>11</v>
+      </c>
+      <c r="D17" t="str">
+        <v>100</v>
+      </c>
+      <c r="E17" t="str">
+        <v>80</v>
+      </c>
+      <c r="F17" t="str">
+        <v>20</v>
+      </c>
+      <c r="G17" t="str">
+        <v>8.8</v>
+      </c>
+      <c r="H17" t="str">
+        <v>91.2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Dezembro</v>
+      </c>
+      <c r="B18" t="str">
+        <v>2024</v>
+      </c>
+      <c r="C18" t="str">
+        <v>12</v>
+      </c>
+      <c r="D18" t="str">
+        <v>100</v>
+      </c>
+      <c r="E18" t="str">
+        <v>80</v>
+      </c>
+      <c r="F18" t="str">
+        <v>20</v>
+      </c>
+      <c r="G18" t="str">
+        <v>8.8</v>
+      </c>
+      <c r="H18" t="str">
+        <v>91.2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Janeiro</v>
+      </c>
+      <c r="B19" t="str">
+        <v>2025</v>
+      </c>
+      <c r="C19" t="str">
+        <v>13</v>
+      </c>
+      <c r="D19" t="str">
+        <v>100</v>
+      </c>
+      <c r="E19" t="str">
+        <v>80</v>
+      </c>
+      <c r="F19" t="str">
+        <v>20</v>
+      </c>
+      <c r="G19" t="str">
+        <v>8.8</v>
+      </c>
+      <c r="H19" t="str">
+        <v>91.2</v>
       </c>
     </row>
     <row r="22">

</xml_diff>